<commit_message>
Analyst Awakening: 52w high is an upweight, not a gate; re-render all books
The archetype now fires on conviction (rating <= 2.2 AND upside >= 25% or
breadth >= 5, >= 3 analysts) plus not-extended, with the fresh-52w-high-
from-base as the top-weighted score component (0.30) instead of a hard
requirement — 1,788 names vs 59, tape-confirmed names ranked first.
All books re-rendered on the fixed propagation + reworked gate.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Pk8K7QpC1m36MYjRwkTznS
</commit_message>
<xml_diff>
--- a/top_n_otc.xlsx
+++ b/top_n_otc.xlsx
@@ -969,7 +969,7 @@
         <v>0.2824096008554864</v>
       </c>
       <c r="C11" s="13" t="n">
-        <v>0.2924482618098654</v>
+        <v>0.2926315239180217</v>
       </c>
       <c r="E11" s="13" t="n">
         <v>1.163700926871588</v>
@@ -1989,26 +1989,26 @@
       </c>
       <c r="B29" s="11" t="inlineStr">
         <is>
-          <t>GLPGF</t>
+          <t>NXCLF</t>
         </is>
       </c>
       <c r="C29" s="8" t="inlineStr">
         <is>
-          <t>Lakefront Biotherapeutics</t>
+          <t>LIFULL Co., Ltd.</t>
         </is>
       </c>
       <c r="D29" s="16" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Communication Services</t>
         </is>
       </c>
       <c r="E29" s="9" t="inlineStr">
         <is>
-          <t>Mid Cap</t>
+          <t>Small Cap</t>
         </is>
       </c>
       <c r="F29" s="10" t="n">
-        <v>3189103616</v>
+        <v>202778128</v>
       </c>
       <c r="G29" s="17" t="inlineStr">
         <is>
@@ -2016,46 +2016,48 @@
         </is>
       </c>
       <c r="H29" s="18" t="n">
-        <v>0.881989217820347</v>
+        <v>0.8938697664316019</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>0.5877493536277286</v>
+        <v>0.5358060628784111</v>
       </c>
       <c r="J29" s="12" t="n">
-        <v>0.5358009711298616</v>
+        <v>0.2390220859642449</v>
       </c>
       <c r="K29" s="12" t="n">
-        <v>4.6826925</v>
+        <v>9.875000999999999</v>
       </c>
       <c r="L29" s="19" t="n">
-        <v>0.9802465124613901</v>
-      </c>
-      <c r="M29" s="20" t="n">
-        <v>-9.730978900874939</v>
+        <v>0.0074367597462133</v>
+      </c>
+      <c r="M29" s="24" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
       <c r="N29" s="20" t="n">
-        <v>214.8679223530429</v>
+        <v>14.40111736061304</v>
       </c>
       <c r="O29" s="19" t="n">
-        <v>-7.475150278954917</v>
+        <v>0.200456447318372</v>
       </c>
       <c r="P29" s="20" t="n">
-        <v>38.14057362285293</v>
+        <v>18.69378177551818</v>
       </c>
       <c r="Q29" s="20" t="n">
-        <v>-8.347884944836451</v>
+        <v>31.55704209289034</v>
       </c>
       <c r="R29" s="21" t="n">
-        <v>0.6458697123620912</v>
+        <v>0.5131200055934176</v>
       </c>
       <c r="S29" s="22" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="T29" s="21" t="n">
-        <v>0.625</v>
+        <v>1</v>
       </c>
       <c r="U29" s="21" t="n">
-        <v>3.055422759429443</v>
+        <v>0.0072093763287943</v>
       </c>
     </row>
     <row r="30" ht="16" customHeight="1">
@@ -2064,17 +2066,17 @@
       </c>
       <c r="B30" s="11" t="inlineStr">
         <is>
-          <t>VTSYF</t>
+          <t>GLPGF</t>
         </is>
       </c>
       <c r="C30" s="8" t="inlineStr">
         <is>
-          <t>Vitasoy International Holdings Limited</t>
+          <t>Lakefront Biotherapeutics</t>
         </is>
       </c>
       <c r="D30" s="16" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
@@ -2083,7 +2085,7 @@
         </is>
       </c>
       <c r="F30" s="10" t="n">
-        <v>803658432</v>
+        <v>3189103616</v>
       </c>
       <c r="G30" s="17" t="inlineStr">
         <is>
@@ -2091,46 +2093,46 @@
         </is>
       </c>
       <c r="H30" s="18" t="n">
-        <v>0.8808517979838447</v>
+        <v>0.881989217820347</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>0.5111983023788198</v>
+        <v>0.5877493536277286</v>
       </c>
       <c r="J30" s="12" t="n">
-        <v>0.2022806204753344</v>
+        <v>0.5358009711298616</v>
       </c>
       <c r="K30" s="12" t="n">
-        <v>26.333334</v>
+        <v>4.6826925</v>
       </c>
       <c r="L30" s="19" t="n">
-        <v>0.277008686396643</v>
+        <v>0.9802465124613901</v>
       </c>
       <c r="M30" s="20" t="n">
-        <v>69.75052804522805</v>
+        <v>-9.730978900874939</v>
       </c>
       <c r="N30" s="20" t="n">
-        <v>14.19375766373652</v>
+        <v>214.8679223530429</v>
       </c>
       <c r="O30" s="19" t="n">
-        <v>-0.7997894533258902</v>
+        <v>-7.475150278954917</v>
       </c>
       <c r="P30" s="20" t="n">
-        <v>15.01383812161213</v>
+        <v>38.14057362285293</v>
       </c>
       <c r="Q30" s="20" t="n">
-        <v>-30.5390929037204</v>
+        <v>-8.347884944836451</v>
       </c>
       <c r="R30" s="21" t="n">
-        <v>0.9897038473558776</v>
+        <v>0.6458697123620912</v>
       </c>
       <c r="S30" s="22" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="T30" s="21" t="n">
-        <v>1</v>
+        <v>0.625</v>
       </c>
       <c r="U30" s="21" t="n">
-        <v>0.1325916317929503</v>
+        <v>3.055422759429443</v>
       </c>
     </row>
     <row r="31" ht="16" customHeight="1">
@@ -2139,26 +2141,26 @@
       </c>
       <c r="B31" s="11" t="inlineStr">
         <is>
-          <t>AKRTF</t>
+          <t>VTSYF</t>
         </is>
       </c>
       <c r="C31" s="8" t="inlineStr">
         <is>
-          <t>Aker Solutions ASA</t>
+          <t>Vitasoy International Holdings Limited</t>
         </is>
       </c>
       <c r="D31" s="16" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="E31" s="9" t="inlineStr">
         <is>
-          <t>Small Cap</t>
+          <t>Mid Cap</t>
         </is>
       </c>
       <c r="F31" s="10" t="n">
-        <v>2162934272</v>
+        <v>803658432</v>
       </c>
       <c r="G31" s="17" t="inlineStr">
         <is>
@@ -2166,46 +2168,46 @@
         </is>
       </c>
       <c r="H31" s="18" t="n">
-        <v>0.8756363829574741</v>
+        <v>0.8808517979838447</v>
       </c>
       <c r="I31" s="12" t="n">
-        <v>0.5740475914015073</v>
+        <v>0.5111983023788198</v>
       </c>
       <c r="J31" s="12" t="n">
-        <v>0.1002714467046379</v>
+        <v>0.2022806204753344</v>
       </c>
       <c r="K31" s="12" t="n">
-        <v>6.357143</v>
+        <v>26.333334</v>
       </c>
       <c r="L31" s="19" t="n">
-        <v>0.1899476834987266</v>
+        <v>0.277008686396643</v>
       </c>
       <c r="M31" s="20" t="n">
-        <v>97.83006480559388</v>
+        <v>69.75052804522805</v>
       </c>
       <c r="N31" s="20" t="n">
-        <v>29.09419471425344</v>
+        <v>14.19375766373652</v>
       </c>
       <c r="O31" s="19" t="n">
-        <v>-0.5152563059397884</v>
+        <v>-0.7997894533258902</v>
       </c>
       <c r="P31" s="20" t="n">
-        <v>7.903282852641389</v>
+        <v>15.01383812161213</v>
       </c>
       <c r="Q31" s="20" t="n">
-        <v>48.68024603713753</v>
+        <v>-30.5390929037204</v>
       </c>
       <c r="R31" s="21" t="n">
-        <v>0.6682729016026684</v>
+        <v>0.9897038473558776</v>
       </c>
       <c r="S31" s="22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T31" s="21" t="n">
         <v>1</v>
       </c>
       <c r="U31" s="21" t="n">
-        <v>0.0347727447992026</v>
+        <v>0.1325916317929503</v>
       </c>
     </row>
     <row r="32" ht="16" customHeight="1">
@@ -2214,17 +2216,17 @@
       </c>
       <c r="B32" s="11" t="inlineStr">
         <is>
-          <t>NXCLF</t>
+          <t>AKRTF</t>
         </is>
       </c>
       <c r="C32" s="8" t="inlineStr">
         <is>
-          <t>LIFULL Co., Ltd.</t>
+          <t>Aker Solutions ASA</t>
         </is>
       </c>
       <c r="D32" s="16" t="inlineStr">
         <is>
-          <t>Communication Services</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">
@@ -2233,7 +2235,7 @@
         </is>
       </c>
       <c r="F32" s="10" t="n">
-        <v>202778128</v>
+        <v>2162934272</v>
       </c>
       <c r="G32" s="17" t="inlineStr">
         <is>
@@ -2241,48 +2243,46 @@
         </is>
       </c>
       <c r="H32" s="18" t="n">
-        <v>0.8752474796309435</v>
+        <v>0.8756363829574741</v>
       </c>
       <c r="I32" s="12" t="n">
-        <v>0.5358060628784111</v>
+        <v>0.5740475914015073</v>
       </c>
       <c r="J32" s="12" t="n">
-        <v>0.2390220859642449</v>
+        <v>0.1002714467046379</v>
       </c>
       <c r="K32" s="12" t="n">
-        <v>9.875000999999999</v>
+        <v>6.357143</v>
       </c>
       <c r="L32" s="19" t="n">
-        <v>0.0074367597462133</v>
-      </c>
-      <c r="M32" s="24" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+        <v>0.1899476834987266</v>
+      </c>
+      <c r="M32" s="20" t="n">
+        <v>97.83006480559388</v>
       </c>
       <c r="N32" s="20" t="n">
-        <v>14.40111736061304</v>
+        <v>29.09419471425344</v>
       </c>
       <c r="O32" s="19" t="n">
-        <v>0.200456447318372</v>
+        <v>-0.5152563059397884</v>
       </c>
       <c r="P32" s="20" t="n">
-        <v>18.69378177551818</v>
+        <v>7.903282852641389</v>
       </c>
       <c r="Q32" s="20" t="n">
-        <v>31.55704209289034</v>
+        <v>48.68024603713753</v>
       </c>
       <c r="R32" s="21" t="n">
-        <v>0.5131200055934176</v>
+        <v>0.6682729016026684</v>
       </c>
       <c r="S32" s="22" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="T32" s="21" t="n">
-        <v>0.875</v>
+        <v>1</v>
       </c>
       <c r="U32" s="21" t="n">
-        <v>0.0072093763287943</v>
+        <v>0.0347727447992026</v>
       </c>
     </row>
     <row r="33" ht="16" customHeight="1">
@@ -2780,7 +2780,7 @@
         </is>
       </c>
       <c r="H39" s="18" t="n">
-        <v>0.8484462743863785</v>
+        <v>0.8425071504656739</v>
       </c>
       <c r="I39" s="12" t="n">
         <v>0.4713590413257659</v>
@@ -2818,7 +2818,7 @@
         <v>3</v>
       </c>
       <c r="T39" s="21" t="n">
-        <v>0.875</v>
+        <v>0.833</v>
       </c>
       <c r="U39" s="21" t="n">
         <v>0.0112918851891152</v>

</xml_diff>